<commit_message>
Corrige el comentario sobre comparabilidad de indicadores de pobreza
Quita la narración del indicador descartado (tasa de pobreza por
líneas nacionales del Banco Mundial) y deja solo lo que importa: los
indicadores de contexto deben ser comparables entre países/regiones.
</commit_message>
<xml_diff>
--- a/SelecciónDatasetsProyecto/INFORME_PISA/INFORME_PISA_metadatos.xlsx
+++ b/SelecciónDatasetsProyecto/INFORME_PISA/INFORME_PISA_metadatos.xlsx
@@ -479,7 +479,7 @@
     <t xml:space="preserve">índice 0-100</t>
   </si>
   <si>
-    <t xml:space="preserve">Desigualdad de ingresos (0 = igualdad perfecta, 100 = desigualdad máxima). Diseñado explícitamente para comparar ENTRE países, al contrario que la tasa de pobreza por líneas nacionales (descartada, ver nota abajo). Mide desigualdad de la DISTRIBUCIÓN, no pobreza en sí. Comprobado con datos reales: Noruega/Finlandia ~26-27, España ~33, Brasil/Sudáfrica ~50-54.</t>
+    <t xml:space="preserve">Desigualdad de ingresos (0 = igualdad perfecta, 100 = desigualdad máxima). Diseñado explícitamente para comparar ENTRE países. Mide desigualdad de la DISTRIBUCIÓN, no pobreza en sí. Comprobado con datos reales: Noruega/Finlandia ~26-27, España ~33, Brasil/Sudáfrica ~50-54.</t>
   </si>
   <si>
     <t xml:space="preserve">pobreza_relativa_pct</t>
@@ -491,7 +491,7 @@
     <t xml:space="preserve">% de población</t>
   </si>
   <si>
-    <t xml:space="preserve">Pobreza RELATIVA: % de población con renta por debajo del 50% de la renta mediana de su propio país (estándar tipo OCDE). A diferencia de la tasa por líneas NACIONALES (descartada), el umbral se calcula igual en todos los países, así que sí es comparable entre ellos, y a diferencia del Gini mide pobreza propiamente, no desigualdad. Comprobado con datos reales: Finlandia/Noruega ~7%, España ~15%, Brasil/Sudáfrica ~20-21% (correlación con indice_gini = 0,84: relacionados pero no redundantes).</t>
+    <t xml:space="preserve">Pobreza RELATIVA: % de población con renta por debajo del 50% de la renta mediana de su propio país (estándar tipo OCDE). El umbral se calcula igual en todos los países, así que es comparable entre ellos, y a diferencia del Gini mide pobreza propiamente, no desigualdad. Comprobado con datos reales: Finlandia/Noruega ~7%, España ~15%, Brasil/Sudáfrica ~20-21% (correlación con indice_gini = 0,84: relacionados pero no redundantes).</t>
   </si>
   <si>
     <t xml:space="preserve">pobreza_pct</t>
@@ -503,7 +503,7 @@
     <t xml:space="preserve">INE, Encuesta de Condiciones de Vida (ECV)</t>
   </si>
   <si>
-    <t xml:space="preserve">Tasa de riesgo de pobreza (renta del año anterior a la entrevista), sin alquiler imputado. Misma encuesta y el mismo umbral metodológico en las 19 CCAA: comparable entre regiones (no tiene el problema de 'línea nacional' propio de comparar entre países distintos).</t>
+    <t xml:space="preserve">Tasa de riesgo de pobreza (renta del año anterior a la entrevista), sin alquiler imputado. Misma encuesta y el mismo umbral metodológico en las 19 CCAA: comparable entre regiones.</t>
   </si>
   <si>
     <t xml:space="preserve">arope_pct</t>

</xml_diff>